<commit_message>
feat(admin): add seller performance, review analysis, and dashboard caching
- Create SellerPerformanceController and view for seller revenue chart
- Implement Cache::remember for AdminDashboardController KPI and trends
- Add Refresh Data button to Admin Dashboard
- Create ReviewAnalysisController and moderation feature
- Introduce Category management for products
- Update routes and sidebar navigation for new admin features
</commit_message>
<xml_diff>
--- a/docs/testing/spreadsheet-output/net-profit.xlsx
+++ b/docs/testing/spreadsheet-output/net-profit.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
   <si>
     <t>Tanggal</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Laba Bersih (Rp)</t>
   </si>
   <si>
-    <t>31/12/2099</t>
+    <t>01/01/2099</t>
   </si>
   <si>
     <t>12/07/2026</t>
@@ -38,40 +38,55 @@
     <t>11/07/2026</t>
   </si>
   <si>
-    <t>08/07/2026</t>
-  </si>
-  <si>
-    <t>07/07/2026</t>
-  </si>
-  <si>
-    <t>05/07/2026</t>
+    <t>10/07/2026</t>
+  </si>
+  <si>
+    <t>09/07/2026</t>
+  </si>
+  <si>
+    <t>04/07/2026</t>
   </si>
   <si>
     <t>03/07/2026</t>
   </si>
   <si>
+    <t>02/07/2026</t>
+  </si>
+  <si>
+    <t>01/07/2026</t>
+  </si>
+  <si>
     <t>30/06/2026</t>
   </si>
   <si>
+    <t>29/06/2026</t>
+  </si>
+  <si>
+    <t>28/06/2026</t>
+  </si>
+  <si>
     <t>26/06/2026</t>
   </si>
   <si>
+    <t>25/06/2026</t>
+  </si>
+  <si>
+    <t>24/06/2026</t>
+  </si>
+  <si>
     <t>22/06/2026</t>
   </si>
   <si>
     <t>21/06/2026</t>
   </si>
   <si>
-    <t>20/06/2026</t>
-  </si>
-  <si>
-    <t>19/06/2026</t>
-  </si>
-  <si>
     <t>17/06/2026</t>
   </si>
   <si>
-    <t>16/06/2026</t>
+    <t>15/06/2026</t>
+  </si>
+  <si>
+    <t>14/06/2026</t>
   </si>
 </sst>
 </file>
@@ -411,7 +426,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
@@ -453,13 +468,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>1024000.0</v>
+        <v>1873000.0</v>
       </c>
       <c r="C3">
         <v>0.0</v>
       </c>
       <c r="D3">
-        <v>1024000.0</v>
+        <v>1873000.0</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -467,13 +482,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>1249000.0</v>
+        <v>2334000.0</v>
       </c>
       <c r="C4">
         <v>0.0</v>
       </c>
       <c r="D4">
-        <v>1249000.0</v>
+        <v>2334000.0</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -481,13 +496,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>1687000.0</v>
+        <v>76000.0</v>
       </c>
       <c r="C5">
         <v>0.0</v>
       </c>
       <c r="D5">
-        <v>1687000.0</v>
+        <v>76000.0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -495,13 +510,13 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>452000.0</v>
+        <v>51000.0</v>
       </c>
       <c r="C6">
         <v>0.0</v>
       </c>
       <c r="D6">
-        <v>452000.0</v>
+        <v>51000.0</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -509,13 +524,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>561000.0</v>
+        <v>46000.0</v>
       </c>
       <c r="C7">
         <v>0.0</v>
       </c>
       <c r="D7">
-        <v>561000.0</v>
+        <v>46000.0</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -523,13 +538,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>856000.0</v>
+        <v>617000.0</v>
       </c>
       <c r="C8">
         <v>0.0</v>
       </c>
       <c r="D8">
-        <v>856000.0</v>
+        <v>617000.0</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -537,13 +552,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1448000.0</v>
+        <v>1708000.0</v>
       </c>
       <c r="C9">
         <v>0.0</v>
       </c>
       <c r="D9">
-        <v>1448000.0</v>
+        <v>1708000.0</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -551,13 +566,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>675000.0</v>
+        <v>655000.0</v>
       </c>
       <c r="C10">
         <v>0.0</v>
       </c>
       <c r="D10">
-        <v>675000.0</v>
+        <v>655000.0</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -565,13 +580,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>245000.0</v>
+        <v>1750000.0</v>
       </c>
       <c r="C11">
         <v>0.0</v>
       </c>
       <c r="D11">
-        <v>245000.0</v>
+        <v>1750000.0</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -579,13 +594,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>1754000.0</v>
+        <v>525000.0</v>
       </c>
       <c r="C12">
         <v>0.0</v>
       </c>
       <c r="D12">
-        <v>1754000.0</v>
+        <v>525000.0</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -593,13 +608,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>1081000.0</v>
+        <v>594000.0</v>
       </c>
       <c r="C13">
         <v>0.0</v>
       </c>
       <c r="D13">
-        <v>1081000.0</v>
+        <v>594000.0</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -607,13 +622,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>1548000.0</v>
+        <v>828000.0</v>
       </c>
       <c r="C14">
         <v>0.0</v>
       </c>
       <c r="D14">
-        <v>1548000.0</v>
+        <v>828000.0</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -621,13 +636,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>1111000.0</v>
+        <v>51000.0</v>
       </c>
       <c r="C15">
         <v>0.0</v>
       </c>
       <c r="D15">
-        <v>1111000.0</v>
+        <v>51000.0</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -635,13 +650,83 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>3003000.0</v>
+        <v>446000.0</v>
       </c>
       <c r="C16">
         <v>0.0</v>
       </c>
       <c r="D16">
-        <v>3003000.0</v>
+        <v>446000.0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>1288000.0</v>
+      </c>
+      <c r="C17">
+        <v>0.0</v>
+      </c>
+      <c r="D17">
+        <v>1288000.0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>278000.0</v>
+      </c>
+      <c r="C18">
+        <v>0.0</v>
+      </c>
+      <c r="D18">
+        <v>278000.0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19">
+        <v>810000.0</v>
+      </c>
+      <c r="C19">
+        <v>0.0</v>
+      </c>
+      <c r="D19">
+        <v>810000.0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20">
+        <v>964000.0</v>
+      </c>
+      <c r="C20">
+        <v>0.0</v>
+      </c>
+      <c r="D20">
+        <v>964000.0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21">
+        <v>324000.0</v>
+      </c>
+      <c r="C21">
+        <v>0.0</v>
+      </c>
+      <c r="D21">
+        <v>324000.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: align db schema and refactor order services
- Add phone_number and address to users migration and model
- Add order_number to orders migration and model
- Create SellerOrderService and refactor SellerOrderController
- Refactor OrderController to use OrderService for status updates
- Update OrderSeeder to include order_number
- Add Playwright E2E tests for buyer orders, payments, reviews, and seller orders
- Update generate-crud.md workflow to include E2E testing steps
</commit_message>
<xml_diff>
--- a/docs/testing/spreadsheet-output/net-profit.xlsx
+++ b/docs/testing/spreadsheet-output/net-profit.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
   <si>
     <t>Tanggal</t>
   </si>
@@ -29,10 +29,19 @@
     <t>Laba Bersih (Rp)</t>
   </si>
   <si>
-    <t>01/01/2099</t>
-  </si>
-  <si>
-    <t>12/07/2026</t>
+    <t>17/07/2026</t>
+  </si>
+  <si>
+    <t>16/07/2026</t>
+  </si>
+  <si>
+    <t>15/07/2026</t>
+  </si>
+  <si>
+    <t>14/07/2026</t>
+  </si>
+  <si>
+    <t>13/07/2026</t>
   </si>
   <si>
     <t>11/07/2026</t>
@@ -44,7 +53,10 @@
     <t>09/07/2026</t>
   </si>
   <si>
-    <t>04/07/2026</t>
+    <t>08/07/2026</t>
+  </si>
+  <si>
+    <t>07/07/2026</t>
   </si>
   <si>
     <t>03/07/2026</t>
@@ -53,19 +65,7 @@
     <t>02/07/2026</t>
   </si>
   <si>
-    <t>01/07/2026</t>
-  </si>
-  <si>
-    <t>30/06/2026</t>
-  </si>
-  <si>
-    <t>29/06/2026</t>
-  </si>
-  <si>
-    <t>28/06/2026</t>
-  </si>
-  <si>
-    <t>26/06/2026</t>
+    <t>27/06/2026</t>
   </si>
   <si>
     <t>25/06/2026</t>
@@ -74,19 +74,10 @@
     <t>24/06/2026</t>
   </si>
   <si>
-    <t>22/06/2026</t>
-  </si>
-  <si>
-    <t>21/06/2026</t>
-  </si>
-  <si>
-    <t>17/06/2026</t>
-  </si>
-  <si>
-    <t>15/06/2026</t>
-  </si>
-  <si>
-    <t>14/06/2026</t>
+    <t>23/06/2026</t>
+  </si>
+  <si>
+    <t>18/06/2026</t>
   </si>
 </sst>
 </file>
@@ -426,7 +417,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
@@ -454,13 +445,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>1500000.0</v>
+        <v>346000.0</v>
       </c>
       <c r="C2">
         <v>0.0</v>
       </c>
       <c r="D2">
-        <v>1500000.0</v>
+        <v>346000.0</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -468,13 +459,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>1873000.0</v>
+        <v>909000.0</v>
       </c>
       <c r="C3">
         <v>0.0</v>
       </c>
       <c r="D3">
-        <v>1873000.0</v>
+        <v>909000.0</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -482,13 +473,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>2334000.0</v>
+        <v>232000.0</v>
       </c>
       <c r="C4">
         <v>0.0</v>
       </c>
       <c r="D4">
-        <v>2334000.0</v>
+        <v>232000.0</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -496,13 +487,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>76000.0</v>
+        <v>531000.0</v>
       </c>
       <c r="C5">
         <v>0.0</v>
       </c>
       <c r="D5">
-        <v>76000.0</v>
+        <v>531000.0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -510,13 +501,13 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>51000.0</v>
+        <v>2229000.0</v>
       </c>
       <c r="C6">
         <v>0.0</v>
       </c>
       <c r="D6">
-        <v>51000.0</v>
+        <v>2229000.0</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -524,13 +515,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>46000.0</v>
+        <v>92000.0</v>
       </c>
       <c r="C7">
         <v>0.0</v>
       </c>
       <c r="D7">
-        <v>46000.0</v>
+        <v>92000.0</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -538,13 +529,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>617000.0</v>
+        <v>1736000.0</v>
       </c>
       <c r="C8">
         <v>0.0</v>
       </c>
       <c r="D8">
-        <v>617000.0</v>
+        <v>1736000.0</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -552,13 +543,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1708000.0</v>
+        <v>921000.0</v>
       </c>
       <c r="C9">
         <v>0.0</v>
       </c>
       <c r="D9">
-        <v>1708000.0</v>
+        <v>921000.0</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -566,13 +557,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>655000.0</v>
+        <v>887000.0</v>
       </c>
       <c r="C10">
         <v>0.0</v>
       </c>
       <c r="D10">
-        <v>655000.0</v>
+        <v>887000.0</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -580,13 +571,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>1750000.0</v>
+        <v>2230000.0</v>
       </c>
       <c r="C11">
         <v>0.0</v>
       </c>
       <c r="D11">
-        <v>1750000.0</v>
+        <v>2230000.0</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -594,13 +585,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>525000.0</v>
+        <v>979000.0</v>
       </c>
       <c r="C12">
         <v>0.0</v>
       </c>
       <c r="D12">
-        <v>525000.0</v>
+        <v>979000.0</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -608,13 +599,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>594000.0</v>
+        <v>939000.0</v>
       </c>
       <c r="C13">
         <v>0.0</v>
       </c>
       <c r="D13">
-        <v>594000.0</v>
+        <v>939000.0</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -622,13 +613,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>828000.0</v>
+        <v>551000.0</v>
       </c>
       <c r="C14">
         <v>0.0</v>
       </c>
       <c r="D14">
-        <v>828000.0</v>
+        <v>551000.0</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -636,13 +627,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>51000.0</v>
+        <v>1580000.0</v>
       </c>
       <c r="C15">
         <v>0.0</v>
       </c>
       <c r="D15">
-        <v>51000.0</v>
+        <v>1580000.0</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -650,13 +641,13 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>446000.0</v>
+        <v>1255000.0</v>
       </c>
       <c r="C16">
         <v>0.0</v>
       </c>
       <c r="D16">
-        <v>446000.0</v>
+        <v>1255000.0</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -664,13 +655,13 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>1288000.0</v>
+        <v>1692000.0</v>
       </c>
       <c r="C17">
         <v>0.0</v>
       </c>
       <c r="D17">
-        <v>1288000.0</v>
+        <v>1692000.0</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -678,55 +669,13 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>278000.0</v>
+        <v>2553000.0</v>
       </c>
       <c r="C18">
         <v>0.0</v>
       </c>
       <c r="D18">
-        <v>278000.0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19">
-        <v>810000.0</v>
-      </c>
-      <c r="C19">
-        <v>0.0</v>
-      </c>
-      <c r="D19">
-        <v>810000.0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20">
-        <v>964000.0</v>
-      </c>
-      <c r="C20">
-        <v>0.0</v>
-      </c>
-      <c r="D20">
-        <v>964000.0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21">
-        <v>324000.0</v>
-      </c>
-      <c r="C21">
-        <v>0.0</v>
-      </c>
-      <c r="D21">
-        <v>324000.0</v>
+        <v>2553000.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>